<commit_message>
Rebuild: merged matches (Fornecedores+Unified), re-export eligible workbooks, rebuild rollups and summaries; add explicit terms index and per-file summary; normalize fornecedores (summary + per-sheet)
</commit_message>
<xml_diff>
--- a/Estelita/Processed/Ubem_MusicCueSheet_OriginaisGloboplay_Janeiro24__eligible_with_refs.xlsx
+++ b/Estelita/Processed/Ubem_MusicCueSheet_OriginaisGloboplay_Janeiro24__eligible_with_refs.xlsx
@@ -762,11 +762,11 @@
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr"/>
       <c r="L2" t="n">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>POR SUPUESTO</t>
+          <t>BABY BABY</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -776,16 +776,16 @@
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>IURI RIO BRANCO,MARINA SENA</t>
+          <t>ANDRE LAUDZ,PETER WOLF,SETH JUSTMAN,ZEGON</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>MARINA SENA</t>
+          <t>TROPKILLAZ</t>
         </is>
       </c>
       <c r="Q2" t="n">
-        <v>69</v>
+        <v>50</v>
       </c>
       <c r="R2" t="inlineStr">
         <is>
@@ -795,24 +795,12 @@
       <c r="S2" t="inlineStr"/>
       <c r="T2" t="inlineStr">
         <is>
-          <t>BOA MUSIC RIGHTS,BOA MUSIC RIGHTS</t>
-        </is>
-      </c>
-      <c r="U2" t="inlineStr">
-        <is>
-          <t>MARINA SENA</t>
-        </is>
-      </c>
-      <c r="V2" t="inlineStr">
-        <is>
-          <t>BX7O92000007</t>
-        </is>
-      </c>
-      <c r="W2" t="inlineStr">
-        <is>
-          <t>FULL MIX</t>
-        </is>
-      </c>
+          <t>BMG,WARNER CHAPPELL,WARNER CHAPPELL,BMG</t>
+        </is>
+      </c>
+      <c r="U2" t="inlineStr"/>
+      <c r="V2" t="inlineStr"/>
+      <c r="W2" t="inlineStr"/>
       <c r="X2" t="inlineStr"/>
       <c r="Y2" t="inlineStr"/>
       <c r="Z2" t="inlineStr"/>
@@ -855,7 +843,7 @@
       <c r="J3" t="inlineStr"/>
       <c r="K3" t="inlineStr"/>
       <c r="L3" t="n">
-        <v>25</v>
+        <v>11</v>
       </c>
       <c r="M3" t="inlineStr">
         <is>
@@ -878,7 +866,7 @@
         </is>
       </c>
       <c r="Q3" t="n">
-        <v>28</v>
+        <v>69</v>
       </c>
       <c r="R3" t="inlineStr">
         <is>
@@ -948,11 +936,11 @@
       <c r="J4" t="inlineStr"/>
       <c r="K4" t="inlineStr"/>
       <c r="L4" t="n">
-        <v>1</v>
+        <v>25</v>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>BABY BABY</t>
+          <t>POR SUPUESTO</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
@@ -962,16 +950,16 @@
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>ANDRE LAUDZ,PETER WOLF,SETH JUSTMAN,ZEGON</t>
+          <t>IURI RIO BRANCO,MARINA SENA</t>
         </is>
       </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t>TROPKILLAZ</t>
+          <t>MARINA SENA</t>
         </is>
       </c>
       <c r="Q4" t="n">
-        <v>50</v>
+        <v>28</v>
       </c>
       <c r="R4" t="inlineStr">
         <is>
@@ -981,12 +969,24 @@
       <c r="S4" t="inlineStr"/>
       <c r="T4" t="inlineStr">
         <is>
-          <t>BMG,WARNER CHAPPELL,WARNER CHAPPELL,BMG</t>
-        </is>
-      </c>
-      <c r="U4" t="inlineStr"/>
-      <c r="V4" t="inlineStr"/>
-      <c r="W4" t="inlineStr"/>
+          <t>BOA MUSIC RIGHTS,BOA MUSIC RIGHTS</t>
+        </is>
+      </c>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t>MARINA SENA</t>
+        </is>
+      </c>
+      <c r="V4" t="inlineStr">
+        <is>
+          <t>BX7O92000007</t>
+        </is>
+      </c>
+      <c r="W4" t="inlineStr">
+        <is>
+          <t>FULL MIX</t>
+        </is>
+      </c>
       <c r="X4" t="inlineStr"/>
       <c r="Y4" t="inlineStr"/>
       <c r="Z4" t="inlineStr"/>

</xml_diff>